<commit_message>
fix: correct DIC metric extraction and add absolute fit assessment
- Extract D.bar, pD, DIC correctly from pcnetmeta matrix output
- Add totresdev/n_arms ratio for absolute model fit assessment
- Update .gitignore (devcontainer, .DS_Store)
- Regenerate all analysis outputs with corrected metrics
</commit_message>
<xml_diff>
--- a/output/dpyd_nma_results.xlsx
+++ b/output/dpyd_nma_results.xlsx
@@ -471,7 +471,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>92.2941371281492</v>
+        <v>151.824946526595</v>
       </c>
       <c r="C2" t="n">
         <v>59.5308093984457</v>
@@ -492,7 +492,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>92.03972661997631</v>
+        <v>151.492061756836</v>
       </c>
       <c r="C3" t="n">
         <v>59.4523351368592</v>
@@ -846,7 +846,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -881,7 +881,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>92.29</t>
+          <t>151.82</t>
         </is>
       </c>
     </row>
@@ -900,22 +900,70 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Max_PSRF</t>
+          <t>D.bar</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1.0420</t>
+          <t>92.29</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>totresdev</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>92.29</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>n_arms</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>98</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>totresdev_per_arm</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>0.94</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Max_PSRF</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>1.0420</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>Converged</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
@@ -1260,7 +1308,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1295,7 +1343,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>92.04</t>
+          <t>151.49</t>
         </is>
       </c>
     </row>
@@ -1314,22 +1362,70 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Max_PSRF</t>
+          <t>D.bar</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1.0285</t>
+          <t>92.04</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>totresdev</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>92.04</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>n_arms</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>98</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>totresdev_per_arm</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>0.94</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Max_PSRF</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>1.0285</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>Converged</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>

</xml_diff>

<commit_message>
Remove WT Binary model - consolidate to WT Unified only
- Delete R/model_wt_binary/ directory and compare_models.R
- Remove WT Binary analysis from run_analysis.R and pairwise_analysis.R
- Delete output/wt_binary/ directory and comparison CSVs
- Update README.md to single-model documentation
- Update export_results_xlsx.py to remove binary sheet mappings
- Regenerate dpyd_nma_results.xlsx with unified-only sheets
- Add rank_probabilities.csv to tracked outputs

WT Unified results verified unchanged (hash comparison passed).
</commit_message>
<xml_diff>
--- a/output/dpyd_nma_results.xlsx
+++ b/output/dpyd_nma_results.xlsx
@@ -7,16 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Model Comparison DIC" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Pairwise Probability Results" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Binary Absolute Risks" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Binary Model Summary" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Binary Odds Ratios" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Binary Publication Summary" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Unified Absolute Risks" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Unified Model Summary" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Unified Odds Ratios" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Unified Publication Summary" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Pairwise Probability" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Rank Probabilities" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Absolute Risks" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Model Summary" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Odds Ratios" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Publication Summary" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -434,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -445,192 +441,88 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Dic</t>
+          <t>P 2846 Greater</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Pd</t>
+          <t>P 13 Greater</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Converged</t>
+          <t>Or Ratio Median</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Max Psrf</t>
+          <t>Or Ratio Ci Lower</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Or Ratio Ci Upper</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Interpretation</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>WT Binary</t>
+          <t>binary</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>151.824946526595</v>
+        <v>0.379</v>
       </c>
       <c r="C2" t="n">
-        <v>59.5308093984457</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
+        <v>0.621</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.819</v>
       </c>
       <c r="E2" t="n">
-        <v>1.04203529472073</v>
+        <v>0.239</v>
+      </c>
+      <c r="F2" t="n">
+        <v>3.213</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>13hetho likely more toxic</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>WT Unified</t>
+          <t>unified</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>151.492061756836</v>
+        <v>0.382</v>
       </c>
       <c r="C3" t="n">
-        <v>59.4523351368592</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
+        <v>0.618</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.824</v>
       </c>
       <c r="E3" t="n">
-        <v>1.02853591755022</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Treatment</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Or Vs Reference 95Cri</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Significant</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>P Best</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>WT</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>--</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>--</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>HapB3</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2.0050 (1.2940, 3.1860)</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2846hetho</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>8.2220 (4.5020, 15.5100)</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2Ahetho</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>6.6030 (3.8640, 11.4700)</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>13hetho</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>6.7350 (2.2030, 24.3600)</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
+        <v>0.236</v>
+      </c>
+      <c r="F3" t="n">
+        <v>3.206</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>13hetho likely more toxic</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -643,98 +535,149 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Model</t>
+          <t>Unnamed: 0</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>P 2846 Greater</t>
+          <t>Rank1</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>P 13 Greater</t>
+          <t>Rank2</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Or Ratio Median</t>
+          <t>Rank3</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Or Ratio Ci Lower</t>
+          <t>Rank4</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Or Ratio Ci Upper</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Interpretation</t>
+          <t>Rank5</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>binary</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.379</v>
+        <v>0.9988</v>
       </c>
       <c r="C2" t="n">
-        <v>0.621</v>
+        <v>0.0012</v>
       </c>
       <c r="D2" t="n">
-        <v>0.819</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>0.239</v>
+        <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>3.213</v>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>13hetho likely more toxic</t>
-        </is>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>unified</t>
+          <t>HapB3</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.382</v>
+        <v>0.0008</v>
       </c>
       <c r="C3" t="n">
-        <v>0.618</v>
+        <v>0.979</v>
       </c>
       <c r="D3" t="n">
-        <v>0.824</v>
+        <v>0.0202</v>
       </c>
       <c r="E3" t="n">
-        <v>0.236</v>
+        <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>3.206</v>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>13hetho likely more toxic</t>
-        </is>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2846hetho</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.3601</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.4898</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2Ahetho</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.4026</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.4289</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.1683</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>13hetho</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.0196</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.4271</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.211</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.3419</v>
       </c>
     </row>
   </sheetData>
@@ -748,7 +691,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -766,72 +709,60 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>WT_Clean</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0.2355 (0.1557, 0.3480)</t>
+          <t>0.2681 (0.2158, 0.3319)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>WT_Biased</t>
+          <t>HapB3</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0.2738 (0.2075, 0.3575)</t>
+          <t>0.4245 (0.3353, 0.5186)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>HapB3</t>
+          <t>2846hetho</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0.4280 (0.3379, 0.5238)</t>
+          <t>0.7509 (0.6222, 0.8494)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2846hetho</t>
+          <t>2Ahetho</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0.7495 (0.6200, 0.8476)</t>
+          <t>0.7078 (0.5894, 0.8065)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2Ahetho</t>
+          <t>13hetho</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0.7057 (0.5839, 0.8044)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>13hetho</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>0.7097 (0.4522, 0.8958)</t>
+          <t>0.7117 (0.4537, 0.8970)</t>
         </is>
       </c>
     </row>
@@ -869,7 +800,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>wt_binary</t>
+          <t>wt_unified</t>
         </is>
       </c>
     </row>
@@ -881,7 +812,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>151.82</t>
+          <t>151.49</t>
         </is>
       </c>
     </row>
@@ -893,7 +824,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>59.53</t>
+          <t>59.45</t>
         </is>
       </c>
     </row>
@@ -905,7 +836,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>92.29</t>
+          <t>92.04</t>
         </is>
       </c>
     </row>
@@ -917,7 +848,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>92.29</t>
+          <t>92.04</t>
         </is>
       </c>
     </row>
@@ -953,7 +884,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>1.0420</t>
+          <t>1.0285</t>
         </is>
       </c>
     </row>
@@ -980,7 +911,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -998,7 +929,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>WT_Clean</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1010,60 +941,48 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>WT_Biased</t>
+          <t>HapB3</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1.2190 (0.6520, 2.3260)</t>
+          <t>2.0050 (1.2940, 3.1860)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>HapB3</t>
+          <t>2846hetho</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2.4130 (1.2790, 4.6900)</t>
+          <t>8.2220 (4.5020, 15.5100)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2846hetho</t>
+          <t>2Ahetho</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>9.6880 (4.3930, 21.6300)</t>
+          <t>6.6030 (3.8640, 11.4700)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2Ahetho</t>
+          <t>13hetho</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>7.7340 (3.7490, 16.1700)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>13hetho</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>7.9150 (2.3930, 30.2000)</t>
+          <t>6.7350 (2.2030, 24.3600)</t>
         </is>
       </c>
     </row>
@@ -1078,7 +997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1097,16 +1016,11 @@
           <t>Significant</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>P Best</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>WT_Clean</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1119,35 +1033,33 @@
           <t>--</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>WT_Biased</t>
+          <t>HapB3</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1.2190 (0.6520, 2.3260)</t>
+          <t>2.0050 (1.2940, 3.1860)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>HapB3</t>
+          <t>2846hetho</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2.4130 (1.2790, 4.6900)</t>
+          <t>8.2220 (4.5020, 15.5100)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1155,17 +1067,16 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2846hetho</t>
+          <t>2Ahetho</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>9.6880 (4.3930, 21.6300)</t>
+          <t>6.6030 (3.8640, 11.4700)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1173,347 +1084,21 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2Ahetho</t>
+          <t>13hetho</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>7.7340 (3.7490, 16.1700)</t>
+          <t>6.7350 (2.2030, 24.3600)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
           <t>Yes</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>13hetho</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>7.9150 (2.3930, 30.2000)</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Treatment</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Toxicity Rate</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>WT</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>0.2681 (0.2158, 0.3319)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>HapB3</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>0.4245 (0.3353, 0.5186)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2846hetho</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>0.7509 (0.6222, 0.8494)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2Ahetho</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>0.7078 (0.5894, 0.8065)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>13hetho</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>0.7117 (0.4537, 0.8970)</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Metric</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Model</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>wt_unified</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>DIC</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>151.49</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>pD</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>59.45</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>D.bar</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>92.04</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>totresdev</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>92.04</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>n_arms</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>98</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>totresdev_per_arm</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>0.94</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Max_PSRF</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>1.0285</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Converged</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Treatment</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Or Vs Reference</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>WT</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>--</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>HapB3</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2.0050 (1.2940, 3.1860)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2846hetho</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>8.2220 (4.5020, 15.5100)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2Ahetho</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>6.6030 (3.8640, 11.4700)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>13hetho</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>6.7350 (2.2030, 24.3600)</t>
         </is>
       </c>
     </row>

</xml_diff>